<commit_message>
[FIX] Smote in inference pipelines
</commit_message>
<xml_diff>
--- a/results/metrics_modelling2_filtered_optuna.xlsx
+++ b/results/metrics_modelling2_filtered_optuna.xlsx
@@ -1647,19 +1647,19 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.92</v>
       </c>
       <c r="F34" t="n">
-        <v>0.8717948717948718</v>
+        <v>0.85</v>
       </c>
       <c r="G34" t="n">
-        <v>0.8947368421052632</v>
+        <v>0.85</v>
       </c>
       <c r="H34" t="n">
         <v>0.85</v>
       </c>
       <c r="I34" t="n">
-        <v>0.9068181818181819</v>
+        <v>0.8977272727272728</v>
       </c>
       <c r="J34" t="n">
         <v>1</v>
@@ -1685,19 +1685,19 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9066666666666666</v>
       </c>
       <c r="F35" t="n">
-        <v>0.8780487804878048</v>
+        <v>0.8372093023255814</v>
       </c>
       <c r="G35" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.7826086956521739</v>
       </c>
       <c r="H35" t="n">
         <v>0.9</v>
       </c>
       <c r="I35" t="n">
-        <v>0.9227272727272726</v>
+        <v>0.9045454545454544</v>
       </c>
       <c r="J35" t="n">
         <v>1</v>
@@ -1723,19 +1723,19 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0.8933333333333333</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="F36" t="n">
-        <v>0.8260869565217392</v>
+        <v>0.8780487804878048</v>
       </c>
       <c r="G36" t="n">
-        <v>0.7307692307692307</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="H36" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="I36" t="n">
-        <v>0.9113636363636364</v>
+        <v>0.9227272727272726</v>
       </c>
       <c r="J36" t="n">
         <v>1</v>
@@ -1799,19 +1799,19 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.88</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="F38" t="n">
-        <v>0.7906976744186046</v>
+        <v>0.761904761904762</v>
       </c>
       <c r="G38" t="n">
-        <v>0.7391304347826086</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="H38" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="I38" t="n">
-        <v>0.8704545454545455</v>
+        <v>0.8454545454545455</v>
       </c>
       <c r="J38" t="n">
         <v>1</v>
@@ -2027,19 +2027,19 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.9066666666666666</v>
+        <v>0.8933333333333333</v>
       </c>
       <c r="F44" t="n">
-        <v>0.8205128205128205</v>
+        <v>0.8000000000000002</v>
       </c>
       <c r="G44" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.8</v>
       </c>
       <c r="H44" t="n">
         <v>0.8</v>
       </c>
       <c r="I44" t="n">
-        <v>0.8727272727272728</v>
+        <v>0.8636363636363636</v>
       </c>
       <c r="J44" t="n">
         <v>1</v>
@@ -2144,16 +2144,16 @@
         <v>0.9333333333333333</v>
       </c>
       <c r="F47" t="n">
-        <v>0.8780487804878048</v>
+        <v>0.8717948717948718</v>
       </c>
       <c r="G47" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="H47" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="I47" t="n">
-        <v>0.9227272727272726</v>
+        <v>0.9068181818181819</v>
       </c>
       <c r="J47" t="n">
         <v>1</v>
@@ -2220,16 +2220,16 @@
         <v>0.88</v>
       </c>
       <c r="F49" t="n">
-        <v>0.9072164948453607</v>
+        <v>0.9052631578947369</v>
       </c>
       <c r="G49" t="n">
-        <v>0.8979591836734694</v>
+        <v>0.9148936170212766</v>
       </c>
       <c r="H49" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.8958333333333334</v>
       </c>
       <c r="I49" t="n">
-        <v>0.8657407407407407</v>
+        <v>0.8738425925925927</v>
       </c>
       <c r="J49" t="n">
         <v>1</v>
@@ -2331,19 +2331,19 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>0.88</v>
+        <v>0.8933333333333333</v>
       </c>
       <c r="F52" t="n">
-        <v>0.9052631578947369</v>
+        <v>0.9183673469387755</v>
       </c>
       <c r="G52" t="n">
-        <v>0.9148936170212766</v>
+        <v>0.9</v>
       </c>
       <c r="H52" t="n">
-        <v>0.8958333333333334</v>
+        <v>0.9375</v>
       </c>
       <c r="I52" t="n">
-        <v>0.8738425925925927</v>
+        <v>0.8761574074074074</v>
       </c>
       <c r="J52" t="n">
         <v>1</v>
@@ -2407,19 +2407,19 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>0.8533333333333334</v>
+        <v>0.88</v>
       </c>
       <c r="F54" t="n">
-        <v>0.8865979381443299</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="G54" t="n">
-        <v>0.8775510204081632</v>
+        <v>0.8823529411764706</v>
       </c>
       <c r="H54" t="n">
-        <v>0.8958333333333334</v>
+        <v>0.9375</v>
       </c>
       <c r="I54" t="n">
-        <v>0.8368055555555556</v>
+        <v>0.8576388888888888</v>
       </c>
       <c r="J54" t="n">
         <v>1</v>
@@ -2445,19 +2445,19 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>0.8533333333333334</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="F55" t="n">
-        <v>0.8910891089108911</v>
+        <v>0.9</v>
       </c>
       <c r="G55" t="n">
-        <v>0.8490566037735849</v>
+        <v>0.8653846153846154</v>
       </c>
       <c r="H55" t="n">
         <v>0.9375</v>
       </c>
       <c r="I55" t="n">
-        <v>0.8206018518518519</v>
+        <v>0.8391203703703703</v>
       </c>
       <c r="J55" t="n">
         <v>1</v>
@@ -2483,19 +2483,19 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>0.8533333333333334</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="F56" t="n">
-        <v>0.8910891089108911</v>
+        <v>0.9</v>
       </c>
       <c r="G56" t="n">
-        <v>0.8490566037735849</v>
+        <v>0.8653846153846154</v>
       </c>
       <c r="H56" t="n">
         <v>0.9375</v>
       </c>
       <c r="I56" t="n">
-        <v>0.8206018518518519</v>
+        <v>0.8391203703703703</v>
       </c>
       <c r="J56" t="n">
         <v>1</v>
@@ -2597,19 +2597,19 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0.8133333333333334</v>
+        <v>0.8266666666666667</v>
       </c>
       <c r="F59" t="n">
-        <v>0.8653846153846154</v>
+        <v>0.8737864077669902</v>
       </c>
       <c r="G59" t="n">
-        <v>0.8035714285714286</v>
+        <v>0.8181818181818182</v>
       </c>
       <c r="H59" t="n">
         <v>0.9375</v>
       </c>
       <c r="I59" t="n">
-        <v>0.7650462962962963</v>
+        <v>0.7835648148148149</v>
       </c>
       <c r="J59" t="n">
         <v>1</v>
@@ -2635,19 +2635,19 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>0.84</v>
+        <v>0.8533333333333334</v>
       </c>
       <c r="F60" t="n">
-        <v>0.8799999999999999</v>
+        <v>0.888888888888889</v>
       </c>
       <c r="G60" t="n">
-        <v>0.8461538461538461</v>
+        <v>0.8627450980392157</v>
       </c>
       <c r="H60" t="n">
         <v>0.9166666666666666</v>
       </c>
       <c r="I60" t="n">
-        <v>0.8101851851851851</v>
+        <v>0.8287037037037036</v>
       </c>
       <c r="J60" t="n">
         <v>1</v>

</xml_diff>